<commit_message>
Add register and login stories and refine TA backlog
</commit_message>
<xml_diff>
--- a/TA backlog.xlsx
+++ b/TA backlog.xlsx
@@ -4,17 +4,30 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28260" windowHeight="12660"/>
+    <workbookView windowWidth="24240" windowHeight="11480"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>Story ID</t>
   </si>
@@ -49,6 +62,32 @@
     <t>S1.1</t>
   </si>
   <si>
+    <t>Register Account</t>
+  </si>
+  <si>
+    <t>As a TA, I want to register an account, so that I can use the system to apply for TA positions.</t>
+  </si>
+  <si>
+    <t>1. TA can create an account using required personal information. 2. The account data is saved and can be used for future login.</t>
+  </si>
+  <si>
+    <t>S1.2</t>
+  </si>
+  <si>
+    <t>Login</t>
+  </si>
+  <si>
+    <t>As a TA, I want to log in to the system, so that I can access my profile and applications.</t>
+  </si>
+  <si>
+    <t>1. TA can log in using a valid account and password.
+2. Invalid login attempts show an error message.
+3. TA can access personal functions after login.</t>
+  </si>
+  <si>
+    <t>S1.3</t>
+  </si>
+  <si>
     <t>Applicant Profile</t>
   </si>
   <si>
@@ -58,7 +97,7 @@
     <t>1. Name, ID, and contact saved to text/JSON file.            2. Data can be reloaded on login.</t>
   </si>
   <si>
-    <t>S1.2</t>
+    <t>S1.4</t>
   </si>
   <si>
     <t>CV Upload</t>
@@ -70,7 +109,7 @@
     <t>1. Support for .txt or .pdf files.                     2. File path is linked to the applicant's profile record.</t>
   </si>
   <si>
-    <t>S1.3</t>
+    <t>S1.5</t>
   </si>
   <si>
     <t>Job Search</t>
@@ -82,7 +121,7 @@
     <t>1. System reads and displays jobs from the MO's data file.             2. Shows module name and required skills.</t>
   </si>
   <si>
-    <t>S1.4</t>
+    <t>S1.6</t>
   </si>
   <si>
     <t>Apply for Job</t>
@@ -94,7 +133,7 @@
     <t>1. Clicking "Apply" creates a record in the application file.           2. Prevents duplicate applications for the same job.</t>
   </si>
   <si>
-    <t>S1.5</t>
+    <t>S1.7</t>
   </si>
   <si>
     <t>Status Tracking</t>
@@ -106,16 +145,17 @@
     <t>1. Display list of applied jobs with status (Pending/Selected/Rejected).</t>
   </si>
   <si>
-    <t>S1.6</t>
+    <t>S1.8</t>
   </si>
   <si>
     <t>AI Skill Match</t>
   </si>
   <si>
-    <t>As a TA, I want the system to highlight jobs matching my skills, so that I apply effectively.</t>
-  </si>
-  <si>
-    <t>1. Logic compares profile skills with job requirements.              2. Displays a match percentage or "Missing Skills" list.</t>
+    <t>As a TA, I want the system to highlight jobs that match my skills so that I can apply more effectively.</t>
+  </si>
+  <si>
+    <t>1. The system compares TA skills with job requirements.
+2. The system displays a match percentage or missing skills list.</t>
   </si>
 </sst>
 </file>
@@ -128,7 +168,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -138,13 +178,6 @@
     </font>
     <font>
       <sz val="10"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
@@ -628,150 +661,150 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -787,6 +820,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1" readingOrder="1"/>
@@ -1139,8 +1175,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J8"/>
-  <sheetFormatPr defaultColWidth="8.83653846153846" defaultRowHeight="16.8" outlineLevelRow="7"/>
+  <dimension ref="A1:J10"/>
+  <sheetFormatPr defaultColWidth="8.83653846153846" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="9.16346153846154" style="1" customWidth="1"/>
     <col min="2" max="2" width="16.6634615384615" style="1" customWidth="1"/>
@@ -1153,7 +1189,7 @@
     <col min="10" max="10" width="26.3365384615385" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.75" spans="1:10">
+    <row r="1" ht="17" spans="1:10">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1185,7 +1221,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" ht="76.75" spans="1:6">
+    <row r="2" ht="92" spans="1:6">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -1205,7 +1241,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" ht="76.75" spans="1:6">
+    <row r="3" ht="137.75" spans="1:6">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
@@ -1239,13 +1275,13 @@
         <v>1</v>
       </c>
       <c r="E4" s="4">
-        <v>2</v>
-      </c>
-      <c r="F4" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="F4" s="7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="5" ht="92.75" spans="1:6">
+    <row r="5" ht="76.75" spans="1:6">
       <c r="A5" s="1" t="s">
         <v>22</v>
       </c>
@@ -1259,13 +1295,13 @@
         <v>1</v>
       </c>
       <c r="E5" s="4">
-        <v>2</v>
-      </c>
-      <c r="F5" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="F5" s="7" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="6" ht="61.75" spans="1:6">
+    <row r="6" ht="76.75" spans="1:6">
       <c r="A6" s="1" t="s">
         <v>26</v>
       </c>
@@ -1276,12 +1312,12 @@
         <v>28</v>
       </c>
       <c r="D6" s="4">
+        <v>1</v>
+      </c>
+      <c r="E6" s="4">
         <v>2</v>
       </c>
-      <c r="E6" s="4">
-        <v>3</v>
-      </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="7" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1296,18 +1332,58 @@
         <v>32</v>
       </c>
       <c r="D7" s="4">
+        <v>1</v>
+      </c>
+      <c r="E7" s="4">
         <v>2</v>
       </c>
-      <c r="E7" s="4">
+      <c r="F7" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" ht="61.75" spans="1:6">
+      <c r="A8" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="4">
+        <v>2</v>
+      </c>
+      <c r="E8" s="4">
+        <v>3</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" ht="92.75" spans="1:6">
+      <c r="A9" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" s="4">
+        <v>2</v>
+      </c>
+      <c r="E9" s="4">
         <v>4</v>
       </c>
-      <c r="F7" s="6" t="s">
-        <v>33</v>
+      <c r="F9" s="7" t="s">
+        <v>41</v>
       </c>
     </row>
-    <row r="8" spans="2:6">
-      <c r="B8" s="5"/>
-      <c r="F8" s="5"/>
+    <row r="10" spans="2:6">
+      <c r="B10" s="5"/>
+      <c r="F10" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Refine TA backlog and integrate AI stories
</commit_message>
<xml_diff>
--- a/TA backlog.xlsx
+++ b/TA backlog.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
   <si>
     <t>Story ID</t>
   </si>
@@ -156,6 +156,63 @@
   <si>
     <t>1. The system compares TA skills with job requirements.
 2. The system displays a match percentage or missing skills list.</t>
+  </si>
+  <si>
+    <t>AI-based matching feature using resume and job description.</t>
+  </si>
+  <si>
+    <t>S1.9</t>
+  </si>
+  <si>
+    <t>Optimize resume keywords</t>
+  </si>
+  <si>
+    <t>As an TA, I want the AI to optimize my resume keywords based on the job description, so that I have a higher matching score.</t>
+  </si>
+  <si>
+    <t>1. Given I upload my resume and select a target job.
+2. When I click "Optimize Resume", the AI highlights 3-5 missing keywords .
+3. The AI provides suggested phrasing .
+4. I can preview the updated matching score before saving the optimized resume.</t>
+  </si>
+  <si>
+    <t>AI NLP analysis for resume keyword optimization.</t>
+  </si>
+  <si>
+    <t>S1.10</t>
+  </si>
+  <si>
+    <t>Recommend suitable positions</t>
+  </si>
+  <si>
+    <t>As a TA, I want the AI to recommend jobs that match my resume, so that I don’t need to browse all job posts manually.</t>
+  </si>
+  <si>
+    <t>1. Given I complete my resume profile (education, skills, experience).
+2. The AI shows a "Recommended Jobs" section on my homepage with top 5 matches.
+3. Each recommendation includes a "Match Score" (0-100) and a "Best Fit Reason" .
+4. I can click "Not Interested" to remove a recommendation and improve future suggestions.</t>
+  </si>
+  <si>
+    <t>Recommendation system based on resume and job requirements.</t>
+  </si>
+  <si>
+    <t>S1.11</t>
+  </si>
+  <si>
+    <t>Check the skill gap of the target position</t>
+  </si>
+  <si>
+    <t>As a TA, I want the AI to compare my resume skills with a specific job’s required skills and identify gaps, so that I know which skills to improve for this application</t>
+  </si>
+  <si>
+    <t>1. Given I upload my resume and select a target job from the job list.
+2. When I click "Check Skill Gaps", the AI extracts 5-8 core required skills from the job description .
+3. The AI generates a "Skill Gap Report" with 3 categories: "Matched Skills" , "Partially Matched" , "Missing Skills" .
+4. For each missing/partially matched skill, the AI provides 1-2 improvement resources .</t>
+  </si>
+  <si>
+    <t>AI comparison between resume skills and job requirements.</t>
   </si>
 </sst>
 </file>
@@ -168,7 +225,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -182,6 +239,11 @@
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="宋体"/>
+      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -676,135 +738,135 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -818,14 +880,23 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1175,7 +1246,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultColWidth="8.83653846153846" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="9.16346153846154" style="1" customWidth="1"/>
@@ -1231,13 +1302,13 @@
       <c r="C2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="5">
         <v>1</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="5">
         <v>1</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1251,13 +1322,13 @@
       <c r="C3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="5">
         <v>1</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="5">
         <v>1</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="8" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1271,13 +1342,13 @@
       <c r="C4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="5">
         <v>1</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="5">
         <v>1</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="9" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1291,13 +1362,13 @@
       <c r="C5" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="5">
         <v>1</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="5">
         <v>1</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="9" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1311,13 +1382,13 @@
       <c r="C6" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="5">
         <v>1</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="5">
         <v>2</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="9" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1331,13 +1402,13 @@
       <c r="C7" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="5">
         <v>1</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="5">
         <v>2</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="9" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1351,17 +1422,17 @@
       <c r="C8" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="5">
         <v>2</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="5">
         <v>3</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="9" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="9" ht="92.75" spans="1:6">
+    <row r="9" ht="92.75" spans="1:8">
       <c r="A9" s="1" t="s">
         <v>38</v>
       </c>
@@ -1371,19 +1442,87 @@
       <c r="C9" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="5">
         <v>2</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="5">
         <v>4</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="9" t="s">
         <v>41</v>
       </c>
+      <c r="H9" s="1" t="s">
+        <v>42</v>
+      </c>
     </row>
-    <row r="10" spans="2:6">
-      <c r="B10" s="5"/>
-      <c r="F10" s="5"/>
+    <row r="10" ht="264" spans="1:8">
+      <c r="A10" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="7">
+        <v>2</v>
+      </c>
+      <c r="E10" s="7">
+        <v>4</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" ht="352" spans="1:8">
+      <c r="A11" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" s="7">
+        <v>3</v>
+      </c>
+      <c r="E11" s="7">
+        <v>4</v>
+      </c>
+      <c r="F11" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="12" ht="405" spans="1:8">
+      <c r="A12" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12" s="7">
+        <v>2</v>
+      </c>
+      <c r="E12" s="7">
+        <v>4</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>57</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>